<commit_message>
fix: skip app launch if already running to prevent duplicate instances
</commit_message>
<xml_diff>
--- a/tests/vna/reports/excel/test_results.xlsx
+++ b/tests/vna/reports/excel/test_results.xlsx
@@ -493,7 +493,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-04-15 08:56:49</t>
+          <t>2026-04-15 09:33:14</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t>1.21</t>
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr"/>

</xml_diff>